<commit_message>
analysis: tighten Samyang valuation dates and equity-base controls
</commit_message>
<xml_diff>
--- a/model/DCF_model.xlsx
+++ b/model/DCF_model.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R63313c61e78d45cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="Rc1613b9bc2924a54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R3c700fe6aa6a4071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" r:id="Rb4ce5704b43b4b5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rfd957db78b424984"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="Rd4677e95083f4f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forecast" sheetId="3" r:id="R69cf1c81aee34081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" r:id="R72c2a1ee67574c7f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -519,15 +519,11 @@
       <x:c r="E2" s="2" t="n"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Valuation date</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-30</x:t>
-        </x:is>
+      <x:c r="A3" s="3" t="str">
+        <x:v>Valuation date / price date</x:v>
+      </x:c>
+      <x:c r="B3" s="3" t="str">
+        <x:v>2026-09-18</x:v>
       </x:c>
       <x:c r="C3" s="2" t="n"/>
       <x:c r="D3" s="3" t="inlineStr">
@@ -900,7 +896,7 @@
         <x:v>Market vintage</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Reference price is 2026-09-18 close; the model header date is 2026-06-30. Do not present both as one synchronized valuation date.</x:v>
+        <x:v>Reference price date is 2026-09-18; latest reported actual period ends 2026-06-30. Keep the two dates separate.</x:v>
       </x:c>
       <x:c r="C13" s="17"/>
       <x:c r="D13" s="17"/>

</xml_diff>